<commit_message>
Mechanical design modified, current mechanical rev is 1
</commit_message>
<xml_diff>
--- a/01_Mechanical_Design/MectoSYS_Proto_BOM_Rev4.xlsx
+++ b/01_Mechanical_Design/MectoSYS_Proto_BOM_Rev4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/920e4c882022e26f/Personal Folder/00_Startup/01_Mectosys_Prototype/00_Git_Repo/01_Mechanical_Design/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/920e4c882022e26f/Personal Folder/00_Startup/00_MectoSYS_Repo/01_Mechanical_Design/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="17" documentId="8_{90E4319E-C89B-42A5-9451-8796C6FDEFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1890D83B-3A58-453F-85DF-89C4D592D445}"/>
+  <xr:revisionPtr revIDLastSave="32" documentId="8_{90E4319E-C89B-42A5-9451-8796C6FDEFFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97A03B61-5AAF-4C33-96F3-4934632B3555}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DED39E1D-C519-45F6-B07F-353D55FF40C1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DED39E1D-C519-45F6-B07F-353D55FF40C1}"/>
   </bookViews>
   <sheets>
     <sheet name="BOM" sheetId="4" r:id="rId1"/>
@@ -22,15 +22,6 @@
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -143,7 +134,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="933" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="943" uniqueCount="360">
   <si>
     <t>Sr No</t>
   </si>
@@ -1331,6 +1322,9 @@
   </si>
   <si>
     <t>Received -OK</t>
+  </si>
+  <si>
+    <t>Received - OK</t>
   </si>
 </sst>
 </file>
@@ -1689,7 +1683,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1793,6 +1787,18 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1820,19 +1826,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2533,7 +2526,7 @@
     <col min="3" max="3" width="29.7109375" customWidth="1"/>
     <col min="4" max="4" width="32.140625" customWidth="1"/>
     <col min="5" max="5" width="9.42578125" customWidth="1"/>
-    <col min="6" max="6" width="14.5703125" style="60" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.5703125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="39" customWidth="1"/>
     <col min="8" max="8" width="15" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.7109375" bestFit="1" customWidth="1"/>
@@ -2577,90 +2570,90 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:49">
-      <c r="A1" s="49" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="49" t="s">
+      <c r="A1" s="53" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="53" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="49" t="s">
+      <c r="C1" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="51" t="s">
+      <c r="D1" s="55" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="49" t="s">
+      <c r="E1" s="53" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="61" t="s">
+      <c r="F1" s="60" t="s">
         <v>356</v>
       </c>
-      <c r="G1" s="52" t="s">
+      <c r="G1" s="56" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="53" t="s">
+      <c r="H1" s="57" t="s">
         <v>340</v>
       </c>
-      <c r="I1" s="54"/>
-      <c r="J1" s="54"/>
-      <c r="K1" s="54"/>
-      <c r="L1" s="54"/>
-      <c r="M1" s="54"/>
-      <c r="N1" s="54"/>
-      <c r="O1" s="55"/>
+      <c r="I1" s="58"/>
+      <c r="J1" s="58"/>
+      <c r="K1" s="58"/>
+      <c r="L1" s="58"/>
+      <c r="M1" s="58"/>
+      <c r="N1" s="58"/>
+      <c r="O1" s="59"/>
       <c r="P1" s="36"/>
-      <c r="Q1" s="53" t="s">
+      <c r="Q1" s="57" t="s">
         <v>341</v>
       </c>
-      <c r="R1" s="54"/>
-      <c r="S1" s="54"/>
-      <c r="T1" s="54"/>
-      <c r="U1" s="54"/>
-      <c r="V1" s="54"/>
-      <c r="W1" s="54"/>
-      <c r="X1" s="55"/>
+      <c r="R1" s="58"/>
+      <c r="S1" s="58"/>
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
+      <c r="V1" s="58"/>
+      <c r="W1" s="58"/>
+      <c r="X1" s="59"/>
       <c r="Y1" s="36"/>
-      <c r="Z1" s="53" t="s">
+      <c r="Z1" s="57" t="s">
         <v>342</v>
       </c>
-      <c r="AA1" s="54"/>
-      <c r="AB1" s="54"/>
-      <c r="AC1" s="54"/>
-      <c r="AD1" s="54"/>
-      <c r="AE1" s="54"/>
-      <c r="AF1" s="54"/>
-      <c r="AG1" s="55"/>
+      <c r="AA1" s="58"/>
+      <c r="AB1" s="58"/>
+      <c r="AC1" s="58"/>
+      <c r="AD1" s="58"/>
+      <c r="AE1" s="58"/>
+      <c r="AF1" s="58"/>
+      <c r="AG1" s="59"/>
       <c r="AH1" s="36"/>
-      <c r="AI1" s="53" t="s">
+      <c r="AI1" s="57" t="s">
         <v>343</v>
       </c>
-      <c r="AJ1" s="54"/>
-      <c r="AK1" s="54"/>
-      <c r="AL1" s="54"/>
-      <c r="AM1" s="54"/>
-      <c r="AN1" s="54"/>
-      <c r="AO1" s="54"/>
-      <c r="AP1" s="55"/>
+      <c r="AJ1" s="58"/>
+      <c r="AK1" s="58"/>
+      <c r="AL1" s="58"/>
+      <c r="AM1" s="58"/>
+      <c r="AN1" s="58"/>
+      <c r="AO1" s="58"/>
+      <c r="AP1" s="59"/>
       <c r="AQ1" s="25"/>
-      <c r="AR1" s="49" t="s">
+      <c r="AR1" s="53" t="s">
         <v>13</v>
       </c>
-      <c r="AS1" s="49" t="s">
+      <c r="AS1" s="53" t="s">
         <v>14</v>
       </c>
-      <c r="AT1" s="49"/>
-      <c r="AU1" s="49"/>
-      <c r="AV1" s="49"/>
-      <c r="AW1" s="49"/>
+      <c r="AT1" s="53"/>
+      <c r="AU1" s="53"/>
+      <c r="AV1" s="53"/>
+      <c r="AW1" s="53"/>
     </row>
     <row r="2" spans="1:49">
-      <c r="A2" s="49"/>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="51"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="62"/>
-      <c r="G2" s="52"/>
+      <c r="A2" s="53"/>
+      <c r="B2" s="53"/>
+      <c r="C2" s="53"/>
+      <c r="D2" s="55"/>
+      <c r="E2" s="53"/>
+      <c r="F2" s="61"/>
+      <c r="G2" s="56"/>
       <c r="H2" s="26" t="s">
         <v>6</v>
       </c>
@@ -2761,12 +2754,12 @@
         <v>12</v>
       </c>
       <c r="AQ2" s="25"/>
-      <c r="AR2" s="49"/>
-      <c r="AS2" s="49"/>
-      <c r="AT2" s="49"/>
-      <c r="AU2" s="49"/>
-      <c r="AV2" s="49"/>
-      <c r="AW2" s="49"/>
+      <c r="AR2" s="53"/>
+      <c r="AS2" s="53"/>
+      <c r="AT2" s="53"/>
+      <c r="AU2" s="53"/>
+      <c r="AV2" s="53"/>
+      <c r="AW2" s="53"/>
     </row>
     <row r="3" spans="1:49">
       <c r="A3" s="4">
@@ -2782,7 +2775,7 @@
         <v>226</v>
       </c>
       <c r="E3" s="21"/>
-      <c r="F3" s="56" t="s">
+      <c r="F3" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G3" s="24"/>
@@ -2892,7 +2885,7 @@
       <c r="E4" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F4" s="57" t="s">
+      <c r="F4" s="48" t="s">
         <v>358</v>
       </c>
       <c r="G4" s="24"/>
@@ -3017,7 +3010,7 @@
       <c r="E5" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F5" s="57" t="s">
+      <c r="F5" s="48" t="s">
         <v>358</v>
       </c>
       <c r="G5" s="24"/>
@@ -3142,7 +3135,7 @@
       <c r="E6" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F6" s="57" t="s">
+      <c r="F6" s="48" t="s">
         <v>358</v>
       </c>
       <c r="G6" s="24"/>
@@ -3267,7 +3260,7 @@
       <c r="E7" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F7" s="57" t="s">
+      <c r="F7" s="48" t="s">
         <v>358</v>
       </c>
       <c r="G7" s="24"/>
@@ -3392,7 +3385,7 @@
       <c r="E8" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F8" s="56" t="s">
+      <c r="F8" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G8" s="24"/>
@@ -3515,7 +3508,7 @@
         <v>250</v>
       </c>
       <c r="E9" s="21"/>
-      <c r="F9" s="56" t="s">
+      <c r="F9" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G9" s="24"/>
@@ -3626,7 +3619,7 @@
         <v>252</v>
       </c>
       <c r="E10" s="21"/>
-      <c r="F10" s="56" t="s">
+      <c r="F10" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G10" s="24"/>
@@ -3739,7 +3732,7 @@
       <c r="E11" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F11" s="57" t="s">
+      <c r="F11" s="48" t="s">
         <v>358</v>
       </c>
       <c r="G11" s="24"/>
@@ -3864,7 +3857,7 @@
       <c r="E12" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F12" s="56" t="s">
+      <c r="F12" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G12" s="24"/>
@@ -3972,7 +3965,7 @@
       <c r="E13" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F13" s="56"/>
+      <c r="F13" s="47"/>
       <c r="G13" s="24"/>
       <c r="H13" s="28" t="s">
         <v>227</v>
@@ -4080,7 +4073,7 @@
       <c r="E14" s="21" t="s">
         <v>240</v>
       </c>
-      <c r="F14" s="56"/>
+      <c r="F14" s="47"/>
       <c r="G14" s="24"/>
       <c r="H14" s="28" t="s">
         <v>227</v>
@@ -4188,7 +4181,7 @@
       <c r="E15" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F15" s="56"/>
+      <c r="F15" s="47"/>
       <c r="G15" s="24"/>
       <c r="H15" s="28" t="s">
         <v>227</v>
@@ -4286,8 +4279,8 @@
         <v>17</v>
       </c>
       <c r="E16" s="21"/>
-      <c r="F16" s="56"/>
-      <c r="G16" s="50" t="s">
+      <c r="F16" s="47"/>
+      <c r="G16" s="54" t="s">
         <v>354</v>
       </c>
       <c r="H16" s="28" t="s">
@@ -4372,8 +4365,8 @@
         <v>21</v>
       </c>
       <c r="E17" s="21"/>
-      <c r="F17" s="56"/>
-      <c r="G17" s="50"/>
+      <c r="F17" s="47"/>
+      <c r="G17" s="54"/>
       <c r="H17" s="28" t="s">
         <v>344</v>
       </c>
@@ -4462,8 +4455,8 @@
         <v>28</v>
       </c>
       <c r="E18" s="21"/>
-      <c r="F18" s="56"/>
-      <c r="G18" s="50"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="54"/>
       <c r="H18" s="28" t="s">
         <v>344</v>
       </c>
@@ -4550,8 +4543,8 @@
         <v>34</v>
       </c>
       <c r="E19" s="21"/>
-      <c r="F19" s="56"/>
-      <c r="G19" s="50"/>
+      <c r="F19" s="47"/>
+      <c r="G19" s="54"/>
       <c r="H19" s="28" t="s">
         <v>344</v>
       </c>
@@ -4642,8 +4635,8 @@
         <v>42</v>
       </c>
       <c r="E20" s="21"/>
-      <c r="F20" s="56"/>
-      <c r="G20" s="50"/>
+      <c r="F20" s="47"/>
+      <c r="G20" s="54"/>
       <c r="H20" s="28" t="s">
         <v>344</v>
       </c>
@@ -4732,8 +4725,8 @@
         <v>48</v>
       </c>
       <c r="E21" s="21"/>
-      <c r="F21" s="56"/>
-      <c r="G21" s="50"/>
+      <c r="F21" s="47"/>
+      <c r="G21" s="54"/>
       <c r="H21" s="28" t="s">
         <v>344</v>
       </c>
@@ -4816,8 +4809,8 @@
         <v>51</v>
       </c>
       <c r="E22" s="21"/>
-      <c r="F22" s="56"/>
-      <c r="G22" s="50"/>
+      <c r="F22" s="47"/>
+      <c r="G22" s="54"/>
       <c r="H22" s="28" t="s">
         <v>344</v>
       </c>
@@ -4906,8 +4899,8 @@
         <v>58</v>
       </c>
       <c r="E23" s="21"/>
-      <c r="F23" s="56"/>
-      <c r="G23" s="50"/>
+      <c r="F23" s="47"/>
+      <c r="G23" s="54"/>
       <c r="H23" s="28" t="s">
         <v>344</v>
       </c>
@@ -4992,8 +4985,8 @@
         <v>63</v>
       </c>
       <c r="E24" s="21"/>
-      <c r="F24" s="56"/>
-      <c r="G24" s="50"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="54"/>
       <c r="H24" s="28" t="s">
         <v>344</v>
       </c>
@@ -5078,8 +5071,8 @@
         <v>68</v>
       </c>
       <c r="E25" s="21"/>
-      <c r="F25" s="56"/>
-      <c r="G25" s="50"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="54"/>
       <c r="H25" s="28" t="s">
         <v>344</v>
       </c>
@@ -5166,8 +5159,8 @@
         <v>72</v>
       </c>
       <c r="E26" s="21"/>
-      <c r="F26" s="56"/>
-      <c r="G26" s="50"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="54"/>
       <c r="H26" s="28" t="s">
         <v>344</v>
       </c>
@@ -5256,8 +5249,8 @@
         <v>75</v>
       </c>
       <c r="E27" s="21"/>
-      <c r="F27" s="56"/>
-      <c r="G27" s="50"/>
+      <c r="F27" s="47"/>
+      <c r="G27" s="54"/>
       <c r="H27" s="28" t="s">
         <v>344</v>
       </c>
@@ -5348,8 +5341,8 @@
         <v>79</v>
       </c>
       <c r="E28" s="21"/>
-      <c r="F28" s="56"/>
-      <c r="G28" s="50"/>
+      <c r="F28" s="47"/>
+      <c r="G28" s="54"/>
       <c r="H28" s="28" t="s">
         <v>344</v>
       </c>
@@ -5438,8 +5431,8 @@
         <v>84</v>
       </c>
       <c r="E29" s="21"/>
-      <c r="F29" s="56"/>
-      <c r="G29" s="50"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="54"/>
       <c r="H29" s="28" t="s">
         <v>344</v>
       </c>
@@ -5530,7 +5523,7 @@
         <v>92</v>
       </c>
       <c r="E30" s="21"/>
-      <c r="F30" s="56"/>
+      <c r="F30" s="47"/>
       <c r="G30" s="24"/>
       <c r="H30" s="28" t="s">
         <v>344</v>
@@ -5640,7 +5633,7 @@
         <v>102</v>
       </c>
       <c r="E31" s="21"/>
-      <c r="F31" s="56"/>
+      <c r="F31" s="47"/>
       <c r="G31" s="24"/>
       <c r="H31" s="28" t="s">
         <v>344</v>
@@ -5750,7 +5743,7 @@
         <v>109</v>
       </c>
       <c r="E32" s="21"/>
-      <c r="F32" s="56"/>
+      <c r="F32" s="47"/>
       <c r="G32" s="24"/>
       <c r="H32" s="28" t="s">
         <v>344</v>
@@ -5854,7 +5847,7 @@
         <v>113</v>
       </c>
       <c r="E33" s="21"/>
-      <c r="F33" s="56"/>
+      <c r="F33" s="47"/>
       <c r="G33" s="24"/>
       <c r="H33" s="28" t="s">
         <v>344</v>
@@ -5962,7 +5955,7 @@
         <v>119</v>
       </c>
       <c r="E34" s="21"/>
-      <c r="F34" s="56"/>
+      <c r="F34" s="47"/>
       <c r="G34" s="24"/>
       <c r="H34" s="28" t="s">
         <v>344</v>
@@ -6070,7 +6063,7 @@
         <v>125</v>
       </c>
       <c r="E35" s="21"/>
-      <c r="F35" s="56"/>
+      <c r="F35" s="47"/>
       <c r="G35" s="24"/>
       <c r="H35" s="28" t="s">
         <v>344</v>
@@ -6178,7 +6171,7 @@
         <v>130</v>
       </c>
       <c r="E36" s="21"/>
-      <c r="F36" s="56"/>
+      <c r="F36" s="47"/>
       <c r="G36" s="24"/>
       <c r="H36" s="28" t="s">
         <v>344</v>
@@ -6286,7 +6279,7 @@
         <v>135</v>
       </c>
       <c r="E37" s="21"/>
-      <c r="F37" s="56"/>
+      <c r="F37" s="47"/>
       <c r="G37" s="24"/>
       <c r="H37" s="28" t="s">
         <v>344</v>
@@ -6386,7 +6379,7 @@
         <v>137</v>
       </c>
       <c r="E38" s="21"/>
-      <c r="F38" s="56"/>
+      <c r="F38" s="47"/>
       <c r="G38" s="24"/>
       <c r="H38" s="28" t="s">
         <v>344</v>
@@ -6486,7 +6479,7 @@
         <v>140</v>
       </c>
       <c r="E39" s="21"/>
-      <c r="F39" s="56"/>
+      <c r="F39" s="47"/>
       <c r="G39" s="24"/>
       <c r="H39" s="28" t="s">
         <v>344</v>
@@ -6586,8 +6579,8 @@
         <v>143</v>
       </c>
       <c r="E40" s="21"/>
-      <c r="F40" s="56"/>
-      <c r="G40" s="50" t="s">
+      <c r="F40" s="47"/>
+      <c r="G40" s="54" t="s">
         <v>354</v>
       </c>
       <c r="H40" s="28" t="s">
@@ -6668,8 +6661,8 @@
         <v>145</v>
       </c>
       <c r="E41" s="21"/>
-      <c r="F41" s="56"/>
-      <c r="G41" s="50"/>
+      <c r="F41" s="47"/>
+      <c r="G41" s="54"/>
       <c r="H41" s="28" t="s">
         <v>344</v>
       </c>
@@ -6748,8 +6741,8 @@
         <v>148</v>
       </c>
       <c r="E42" s="21"/>
-      <c r="F42" s="56"/>
-      <c r="G42" s="50"/>
+      <c r="F42" s="47"/>
+      <c r="G42" s="54"/>
       <c r="H42" s="28" t="s">
         <v>344</v>
       </c>
@@ -6830,8 +6823,8 @@
         <v>150</v>
       </c>
       <c r="E43" s="21"/>
-      <c r="F43" s="56"/>
-      <c r="G43" s="50"/>
+      <c r="F43" s="47"/>
+      <c r="G43" s="54"/>
       <c r="H43" s="28" t="s">
         <v>344</v>
       </c>
@@ -6910,8 +6903,8 @@
         <v>153</v>
       </c>
       <c r="E44" s="21"/>
-      <c r="F44" s="56"/>
-      <c r="G44" s="50"/>
+      <c r="F44" s="47"/>
+      <c r="G44" s="54"/>
       <c r="H44" s="28" t="s">
         <v>344</v>
       </c>
@@ -6990,8 +6983,8 @@
         <v>155</v>
       </c>
       <c r="E45" s="21"/>
-      <c r="F45" s="56"/>
-      <c r="G45" s="50"/>
+      <c r="F45" s="47"/>
+      <c r="G45" s="54"/>
       <c r="H45" s="28" t="s">
         <v>344</v>
       </c>
@@ -7070,8 +7063,8 @@
         <v>158</v>
       </c>
       <c r="E46" s="21"/>
-      <c r="F46" s="56"/>
-      <c r="G46" s="50"/>
+      <c r="F46" s="47"/>
+      <c r="G46" s="54"/>
       <c r="H46" s="28" t="s">
         <v>344</v>
       </c>
@@ -7150,8 +7143,8 @@
         <v>161</v>
       </c>
       <c r="E47" s="21"/>
-      <c r="F47" s="56"/>
-      <c r="G47" s="50"/>
+      <c r="F47" s="47"/>
+      <c r="G47" s="54"/>
       <c r="H47" s="28" t="s">
         <v>344</v>
       </c>
@@ -7228,8 +7221,8 @@
         <v>163</v>
       </c>
       <c r="E48" s="21"/>
-      <c r="F48" s="56"/>
-      <c r="G48" s="50"/>
+      <c r="F48" s="47"/>
+      <c r="G48" s="54"/>
       <c r="H48" s="28" t="s">
         <v>344</v>
       </c>
@@ -7308,8 +7301,8 @@
         <v>165</v>
       </c>
       <c r="E49" s="21"/>
-      <c r="F49" s="56"/>
-      <c r="G49" s="50"/>
+      <c r="F49" s="47"/>
+      <c r="G49" s="54"/>
       <c r="H49" s="28" t="s">
         <v>344</v>
       </c>
@@ -7386,8 +7379,8 @@
         <v>167</v>
       </c>
       <c r="E50" s="21"/>
-      <c r="F50" s="56"/>
-      <c r="G50" s="50"/>
+      <c r="F50" s="47"/>
+      <c r="G50" s="54"/>
       <c r="H50" s="28" t="s">
         <v>344</v>
       </c>
@@ -7464,8 +7457,8 @@
         <v>170</v>
       </c>
       <c r="E51" s="21"/>
-      <c r="F51" s="56"/>
-      <c r="G51" s="50"/>
+      <c r="F51" s="47"/>
+      <c r="G51" s="54"/>
       <c r="H51" s="28" t="s">
         <v>344</v>
       </c>
@@ -7542,8 +7535,8 @@
         <v>172</v>
       </c>
       <c r="E52" s="21"/>
-      <c r="F52" s="56"/>
-      <c r="G52" s="50"/>
+      <c r="F52" s="47"/>
+      <c r="G52" s="54"/>
       <c r="H52" s="28" t="s">
         <v>344</v>
       </c>
@@ -7620,8 +7613,8 @@
         <v>175</v>
       </c>
       <c r="E53" s="21"/>
-      <c r="F53" s="56"/>
-      <c r="G53" s="50"/>
+      <c r="F53" s="47"/>
+      <c r="G53" s="54"/>
       <c r="H53" s="28" t="s">
         <v>344</v>
       </c>
@@ -7698,8 +7691,8 @@
         <v>177</v>
       </c>
       <c r="E54" s="21"/>
-      <c r="F54" s="56"/>
-      <c r="G54" s="50"/>
+      <c r="F54" s="47"/>
+      <c r="G54" s="54"/>
       <c r="H54" s="28" t="s">
         <v>344</v>
       </c>
@@ -7776,8 +7769,8 @@
         <v>179</v>
       </c>
       <c r="E55" s="21"/>
-      <c r="F55" s="56"/>
-      <c r="G55" s="50"/>
+      <c r="F55" s="47"/>
+      <c r="G55" s="54"/>
       <c r="H55" s="28" t="s">
         <v>344</v>
       </c>
@@ -7854,8 +7847,8 @@
         <v>182</v>
       </c>
       <c r="E56" s="21"/>
-      <c r="F56" s="56"/>
-      <c r="G56" s="50"/>
+      <c r="F56" s="47"/>
+      <c r="G56" s="54"/>
       <c r="H56" s="28" t="s">
         <v>344</v>
       </c>
@@ -7930,8 +7923,8 @@
         <v>184</v>
       </c>
       <c r="E57" s="21"/>
-      <c r="F57" s="56"/>
-      <c r="G57" s="50"/>
+      <c r="F57" s="47"/>
+      <c r="G57" s="54"/>
       <c r="H57" s="28" t="s">
         <v>344</v>
       </c>
@@ -8008,7 +8001,7 @@
         <v>187</v>
       </c>
       <c r="E58" s="21"/>
-      <c r="F58" s="56"/>
+      <c r="F58" s="47"/>
       <c r="G58" s="24"/>
       <c r="H58" s="28" t="s">
         <v>344</v>
@@ -8110,7 +8103,9 @@
         <v>190</v>
       </c>
       <c r="E59" s="21"/>
-      <c r="F59" s="56"/>
+      <c r="F59" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G59" s="24"/>
       <c r="H59" s="28" t="s">
         <v>93</v>
@@ -8208,7 +8203,9 @@
         <v>199</v>
       </c>
       <c r="E60" s="21"/>
-      <c r="F60" s="56"/>
+      <c r="F60" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G60" s="24"/>
       <c r="H60" s="28" t="s">
         <v>93</v>
@@ -8304,7 +8301,9 @@
         <v>205</v>
       </c>
       <c r="E61" s="21"/>
-      <c r="F61" s="56"/>
+      <c r="F61" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G61" s="24"/>
       <c r="H61" s="28" t="s">
         <v>93</v>
@@ -8415,7 +8414,9 @@
         <v>214</v>
       </c>
       <c r="E62" s="21"/>
-      <c r="F62" s="56"/>
+      <c r="F62" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G62" s="24"/>
       <c r="H62" s="28" t="s">
         <v>93</v>
@@ -8511,7 +8512,9 @@
         <v>219</v>
       </c>
       <c r="E63" s="21"/>
-      <c r="F63" s="56"/>
+      <c r="F63" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G63" s="24"/>
       <c r="H63" s="28" t="s">
         <v>93</v>
@@ -8607,7 +8610,9 @@
         <v>221</v>
       </c>
       <c r="E64" s="21"/>
-      <c r="F64" s="56"/>
+      <c r="F64" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G64" s="24"/>
       <c r="H64" s="28" t="s">
         <v>93</v>
@@ -8716,7 +8721,9 @@
         <v>223</v>
       </c>
       <c r="E65" s="21"/>
-      <c r="F65" s="56"/>
+      <c r="F65" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G65" s="24"/>
       <c r="H65" s="28" t="s">
         <v>93</v>
@@ -8814,7 +8821,7 @@
         <v>268</v>
       </c>
       <c r="E66" s="21"/>
-      <c r="F66" s="56"/>
+      <c r="F66" s="47"/>
       <c r="G66" s="24" t="s">
         <v>355</v>
       </c>
@@ -8898,7 +8905,7 @@
         <v>271</v>
       </c>
       <c r="E67" s="21"/>
-      <c r="F67" s="56"/>
+      <c r="F67" s="47"/>
       <c r="G67" s="24"/>
       <c r="H67" s="28" t="s">
         <v>349</v>
@@ -9000,7 +9007,7 @@
         <v>274</v>
       </c>
       <c r="E68" s="21"/>
-      <c r="F68" s="56"/>
+      <c r="F68" s="47"/>
       <c r="G68" s="24"/>
       <c r="H68" s="28" t="s">
         <v>349</v>
@@ -9102,7 +9109,7 @@
         <v>277</v>
       </c>
       <c r="E69" s="21"/>
-      <c r="F69" s="56"/>
+      <c r="F69" s="47"/>
       <c r="G69" s="24"/>
       <c r="H69" s="28" t="s">
         <v>349</v>
@@ -9209,7 +9216,7 @@
         <v>280</v>
       </c>
       <c r="E70" s="21"/>
-      <c r="F70" s="56"/>
+      <c r="F70" s="47"/>
       <c r="G70" s="24"/>
       <c r="H70" s="28" t="s">
         <v>349</v>
@@ -9311,7 +9318,7 @@
         <v>283</v>
       </c>
       <c r="E71" s="21"/>
-      <c r="F71" s="56"/>
+      <c r="F71" s="47"/>
       <c r="G71" s="24"/>
       <c r="H71" s="28" t="s">
         <v>349</v>
@@ -9418,7 +9425,7 @@
         <v>286</v>
       </c>
       <c r="E72" s="21"/>
-      <c r="F72" s="56"/>
+      <c r="F72" s="47"/>
       <c r="G72" s="24"/>
       <c r="H72" s="28" t="s">
         <v>349</v>
@@ -9520,8 +9527,8 @@
         <v>289</v>
       </c>
       <c r="E73" s="21"/>
-      <c r="F73" s="58"/>
-      <c r="G73" s="47" t="s">
+      <c r="F73" s="49"/>
+      <c r="G73" s="51" t="s">
         <v>355</v>
       </c>
       <c r="H73" s="28" t="s">
@@ -9604,8 +9611,8 @@
         <v>291</v>
       </c>
       <c r="E74" s="21"/>
-      <c r="F74" s="59"/>
-      <c r="G74" s="48"/>
+      <c r="F74" s="50"/>
+      <c r="G74" s="52"/>
       <c r="H74" s="28" t="s">
         <v>349</v>
       </c>
@@ -9688,7 +9695,7 @@
       <c r="E75" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F75" s="56"/>
+      <c r="F75" s="47"/>
       <c r="G75" s="24"/>
       <c r="H75" s="28" t="s">
         <v>349</v>
@@ -9797,7 +9804,7 @@
         <v>298</v>
       </c>
       <c r="E76" s="21"/>
-      <c r="F76" s="56"/>
+      <c r="F76" s="47"/>
       <c r="G76" s="24"/>
       <c r="H76" s="28" t="s">
         <v>349</v>
@@ -9899,7 +9906,7 @@
         <v>300</v>
       </c>
       <c r="E77" s="21"/>
-      <c r="F77" s="56"/>
+      <c r="F77" s="47"/>
       <c r="G77" s="24"/>
       <c r="H77" s="28" t="s">
         <v>349</v>
@@ -10001,7 +10008,9 @@
         <v>303</v>
       </c>
       <c r="E78" s="21"/>
-      <c r="F78" s="56"/>
+      <c r="F78" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G78" s="24" t="s">
         <v>355</v>
       </c>
@@ -10088,7 +10097,7 @@
         <v>315</v>
       </c>
       <c r="E79" s="21"/>
-      <c r="F79" s="56"/>
+      <c r="F79" s="47"/>
       <c r="G79" s="24"/>
       <c r="H79" s="28" t="s">
         <v>316</v>
@@ -10193,7 +10202,7 @@
         <v>319</v>
       </c>
       <c r="E80" s="21"/>
-      <c r="F80" s="56" t="s">
+      <c r="F80" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G80" s="24" t="s">
@@ -10284,7 +10293,7 @@
         <v>323</v>
       </c>
       <c r="E81" s="21"/>
-      <c r="F81" s="56" t="s">
+      <c r="F81" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G81" s="24" t="s">
@@ -10308,7 +10317,7 @@
       </c>
       <c r="N81" s="6"/>
       <c r="O81" s="29">
-        <f t="shared" ref="O81:O92" si="11">L81*M81</f>
+        <f t="shared" ref="O81:O94" si="11">L81*M81</f>
         <v>33.950000000000003</v>
       </c>
       <c r="P81" s="36"/>
@@ -10370,7 +10379,7 @@
         <v>309</v>
       </c>
       <c r="E82" s="21"/>
-      <c r="F82" s="56" t="s">
+      <c r="F82" s="47" t="s">
         <v>357</v>
       </c>
       <c r="G82" s="24"/>
@@ -10474,7 +10483,7 @@
         <v>312</v>
       </c>
       <c r="E83" s="21"/>
-      <c r="F83" s="56"/>
+      <c r="F83" s="47"/>
       <c r="G83" s="24"/>
       <c r="H83" s="30" t="s">
         <v>95</v>
@@ -10576,7 +10585,9 @@
         <v>326</v>
       </c>
       <c r="E84" s="21"/>
-      <c r="F84" s="56"/>
+      <c r="F84" s="48" t="s">
+        <v>359</v>
+      </c>
       <c r="G84" s="24"/>
       <c r="H84" s="30" t="s">
         <v>328</v>
@@ -10683,7 +10694,7 @@
         <v>332</v>
       </c>
       <c r="E85" s="21"/>
-      <c r="F85" s="56"/>
+      <c r="F85" s="47"/>
       <c r="G85" s="24"/>
       <c r="H85" s="28" t="s">
         <v>333</v>
@@ -10785,7 +10796,7 @@
         <v>336</v>
       </c>
       <c r="E86" s="21"/>
-      <c r="F86" s="56"/>
+      <c r="F86" s="47"/>
       <c r="G86" s="24"/>
       <c r="H86" s="28" t="s">
         <v>333</v>
@@ -10877,7 +10888,9 @@
       <c r="E87" s="21" t="s">
         <v>231</v>
       </c>
-      <c r="F87" s="56"/>
+      <c r="F87" s="47" t="s">
+        <v>357</v>
+      </c>
       <c r="G87" s="24"/>
       <c r="H87" s="28" t="s">
         <v>339</v>
@@ -10982,7 +10995,7 @@
         <v>210</v>
       </c>
       <c r="E88" s="21"/>
-      <c r="F88" s="56"/>
+      <c r="F88" s="47"/>
       <c r="G88" s="24"/>
       <c r="H88" s="30" t="s">
         <v>203</v>
@@ -11082,7 +11095,7 @@
         <v>217</v>
       </c>
       <c r="E89" s="21"/>
-      <c r="F89" s="56"/>
+      <c r="F89" s="47"/>
       <c r="G89" s="24"/>
       <c r="H89" s="30" t="s">
         <v>203</v>
@@ -11182,7 +11195,7 @@
         <v>194</v>
       </c>
       <c r="E90" s="21"/>
-      <c r="F90" s="56"/>
+      <c r="F90" s="47"/>
       <c r="G90" s="24"/>
       <c r="H90" s="30" t="s">
         <v>203</v>
@@ -11282,7 +11295,7 @@
         <v>202</v>
       </c>
       <c r="E91" s="21"/>
-      <c r="F91" s="56"/>
+      <c r="F91" s="47"/>
       <c r="G91" s="24"/>
       <c r="H91" s="30" t="s">
         <v>203</v>
@@ -11380,7 +11393,7 @@
         <v>207</v>
       </c>
       <c r="E92" s="21"/>
-      <c r="F92" s="56"/>
+      <c r="F92" s="47"/>
       <c r="G92" s="24"/>
       <c r="H92" s="31" t="s">
         <v>203</v>

</xml_diff>